<commit_message>
docs: update SPARK_TRACKER.md, SPARK_Component_Order_Form.xlsx - enclosure TPU sourcing switched to 1kg roll purchase (NPR 90->4000, total 9667->13577), Action #37 added, roll vendor TBD
</commit_message>
<xml_diff>
--- a/docs/SPARK_Component_Order_Form.xlsx
+++ b/docs/SPARK_Component_Order_Form.xlsx
@@ -45,7 +45,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">NPR 90 (v38) — hand-computed two-zone geometric estimate from real forearm measurement (12cm/16cm arc, matches render's 75% wrap independently) + DI-01 component footprints, 2mm wall, TPU 1.21 g/cm3. Still NOT a CAD/slicer output — no model exists yet, blocked on Action #17. See tracker Action #36.</t>
+          <t xml:space="preserve">Switched v38 from per-part TPU print-service (KEC Makerspace charges NPR 4/g per print, was NPR 90 for the ~22g enclosure estimate) to buying a 1kg roll outright at the same NPR 4/g rate = NPR 4,000. Team now owns the filament; only ~22g needed for one enclosure per the v38 geometric estimate (tracker Action #36), so most of the roll is spare/future-use, not consumed by this one part. Roll vendor not yet sourced to a live listing — confirm before ordering.</t>
         </r>
       </text>
     </comment>
@@ -161,10 +161,10 @@
     <t xml:space="preserve">Dipen Manandhar (Supervisor)</t>
   </si>
   <si>
-    <t xml:space="preserve">Enclosure (3D-printed TPU, KEC Makerspace)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KEC Makerspace</t>
+    <t xml:space="preserve">TPU filament, 1kg roll (enclosure raw material)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEC Makerspace / vendor TBD</t>
   </si>
   <si>
     <t xml:space="preserve">USB-C cables</t>
@@ -959,11 +959,11 @@
         <v>1</v>
       </c>
       <c r="I11" s="9" t="n">
-        <v>90</v>
+        <v>4000</v>
       </c>
       <c r="J11" s="11" t="n">
         <f aca="false">H11*I11</f>
-        <v>90</v>
+        <v>4000</v>
       </c>
       <c r="K11" s="3"/>
       <c r="L11" s="17"/>
@@ -1083,7 +1083,7 @@
       <c r="I15" s="19"/>
       <c r="J15" s="21" t="n">
         <f aca="false">SUM(J5:J14)</f>
-        <v>9667</v>
+        <v>13577</v>
       </c>
       <c r="K15" s="18"/>
       <c r="L15" s="18"/>

</xml_diff>